<commit_message>
Planilhas de preço oficial por marca
</commit_message>
<xml_diff>
--- a/tools/precos/planilhas/precos-oficiais-Anua.xlsx
+++ b/tools/precos/planilhas/precos-oficiais-Anua.xlsx
@@ -41,12 +41,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E3F4E8"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -72,7 +77,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -81,6 +86,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -582,7 +588,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -635,7 +641,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -690,7 +696,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -745,7 +751,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -800,7 +806,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -853,7 +859,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -906,7 +912,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -959,7 +965,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1014,7 +1020,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1067,7 +1073,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1120,7 +1126,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1173,7 +1179,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1208,12 +1214,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MB003833</t>
+          <t>MB003869</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Breakout Care Duo: sérum de ácido azelaico + creme localizado Heartleaf Centella</t>
+          <t>Collagen Retinol Refining Gua Sha Cream: creme para pescoço com retinol e aplicador 80 ml</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1222,25 +1228,23 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>306.9</v>
+        <v>254.9</v>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Breakout Care Duo</t>
+          <t>Collagen Retinol Refining Gua Sha Cream</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" s="4" t="n">
-        <v>42</v>
-      </c>
-      <c r="I14" s="4" t="n">
-        <v>50</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="I14" s="4" t="n"/>
       <c r="J14" t="inlineStr">
         <is>
           <t>Sim</t>
@@ -1248,7 +1252,7 @@
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/intensive-spot-care-duo</t>
+          <t>https://anua.us/products/collagen-retinol-refining-gua-sha-cream-1</t>
         </is>
       </c>
       <c r="L14" s="2">
@@ -1263,12 +1267,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>MB003869</t>
+          <t>MB002667</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Collagen Retinol Refining Gua Sha Cream: creme para pescoço com retinol e aplicador 80 ml</t>
+          <t>Fall into Deep Hydration Set: rotina viral com PDRN e retinol · Essential Set</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1277,23 +1281,25 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>254.9</v>
+        <v>481.9</v>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Collagen Retinol Refining Gua Sha Cream</t>
+          <t>Fall into Deep Hydration Set</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" s="4" t="n">
-        <v>35</v>
-      </c>
-      <c r="I15" s="4" t="n"/>
+        <v>143</v>
+      </c>
+      <c r="I15" s="4" t="n">
+        <v>210</v>
+      </c>
       <c r="J15" t="inlineStr">
         <is>
           <t>Sim</t>
@@ -1301,7 +1307,7 @@
       </c>
       <c r="K15" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/collagen-retinol-refining-gua-sha-cream-1</t>
+          <t>https://anua.us/products/amazon-x-tiktok-viral-routine-kit</t>
         </is>
       </c>
       <c r="L15" s="2">
@@ -1316,12 +1322,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MB002667</t>
+          <t>MB003823</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Fall into Deep Hydration Set: rotina viral com PDRN e retinol · Essential Set</t>
+          <t>Heartleaf 70 Daily Lotion: loção hidratante leve com heartleaf 200 ml</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1330,25 +1336,23 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>481.9</v>
+        <v>188.9</v>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Fall into Deep Hydration Set</t>
+          <t>Heartleaf 70 Daily Lotion</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" s="4" t="n">
-        <v>143</v>
-      </c>
-      <c r="I16" s="4" t="n">
-        <v>210</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="I16" s="4" t="n"/>
       <c r="J16" t="inlineStr">
         <is>
           <t>Sim</t>
@@ -1356,7 +1360,7 @@
       </c>
       <c r="K16" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/amazon-x-tiktok-viral-routine-kit</t>
+          <t>https://anua.us/products/heartleaf-70-daily-lotion-copy-1</t>
         </is>
       </c>
       <c r="L16" s="2">
@@ -1371,12 +1375,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>MB003823</t>
+          <t>MB003809</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Heartleaf 70 Daily Lotion: loção hidratante leve com heartleaf 200 ml</t>
+          <t>Heartleaf 70% Intense Calming Cream: creme calmante com ceramida 50 ml</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1389,12 +1393,12 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Heartleaf 70 Daily Lotion</t>
+          <t>Heartleaf 70% Intense Calming Cream</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
@@ -1409,7 +1413,7 @@
       </c>
       <c r="K17" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/heartleaf-70-daily-lotion-copy-1</t>
+          <t>https://anua.us/products/heartleaf-70-intense-calming-cream</t>
         </is>
       </c>
       <c r="L17" s="2">
@@ -1424,12 +1428,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>MB003809</t>
+          <t>MB002706</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Heartleaf 70% Intense Calming Cream: creme calmante com ceramida 50 ml</t>
+          <t>Heartleaf 80% Moisture Soothing Ampoule: ampola calmante e hidratante 30 ml</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1438,21 +1442,21 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>188.9</v>
+        <v>159.9</v>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Heartleaf 70% Intense Calming Cream</t>
+          <t>Heartleaf 80% Moisture Soothing Ampoule</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" s="4" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="I18" s="4" t="n"/>
       <c r="J18" t="inlineStr">
@@ -1462,7 +1466,7 @@
       </c>
       <c r="K18" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/heartleaf-70-intense-calming-cream</t>
+          <t>https://anua.us/products/heartleaf-80-moisture-soothing-ampoule-30ml</t>
         </is>
       </c>
       <c r="L18" s="2">
@@ -1477,12 +1481,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MB002706</t>
+          <t>MB003832</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Heartleaf 80% Moisture Soothing Ampoule: ampola calmante e hidratante 30 ml</t>
+          <t>Heartleaf Centella Red Spot Cream: creme calmante para pontinhos vermelhos 30 g</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1491,16 +1495,16 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>159.9</v>
+        <v>160.9</v>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Heartleaf 80% Moisture Soothing Ampoule</t>
+          <t>Heartleaf Centella Red Spot Cream</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
@@ -1515,7 +1519,7 @@
       </c>
       <c r="K19" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/heartleaf-80-moisture-soothing-ampoule-30ml</t>
+          <t>https://anua.us/products/heartleaf-centella-red-spot-cream-1</t>
         </is>
       </c>
       <c r="L19" s="2">
@@ -1530,12 +1534,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MB003832</t>
+          <t>MB003813</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Heartleaf Centella Red Spot Cream: creme calmante para pontinhos vermelhos 30 g</t>
+          <t>Heartleaf LHA Moisture Peeling Gel: gel esfoliante suave com LHA</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1544,16 +1548,16 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>160.9</v>
+        <v>159.9</v>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Heartleaf Centella Red Spot Cream</t>
+          <t>Heartleaf LHA Moisture Peeling Gel</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
@@ -1568,7 +1572,7 @@
       </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/heartleaf-centella-red-spot-cream-1</t>
+          <t>https://anua.us/products/heartleaf-lha-moisture-peeling-gel-copy</t>
         </is>
       </c>
       <c r="L20" s="2">
@@ -1583,12 +1587,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MB003813</t>
+          <t>MB003811</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Heartleaf LHA Moisture Peeling Gel: gel esfoliante suave com LHA</t>
+          <t>Heartleaf Pore Control Cleansing Oil: óleo de limpeza para os poros 200 ml</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1601,12 +1605,12 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Heartleaf LHA Moisture Peeling Gel</t>
+          <t>Heartleaf Pore Control Cleansing Oil</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
@@ -1621,7 +1625,7 @@
       </c>
       <c r="K21" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/heartleaf-lha-moisture-peeling-gel-copy</t>
+          <t>https://anua.us/products/heartleaf-pore-control-cleansing-oil-200ml</t>
         </is>
       </c>
       <c r="L21" s="2">
@@ -1636,12 +1640,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>MB003821</t>
+          <t>MB003871</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Heartleaf Pore Cleansing Oil Mild: óleo de limpeza suave sem fragrância 200 ml</t>
+          <t>Invisible Glow Finish Sunstick: protetor solar em bastão FPS 50 17,5 g</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1650,21 +1654,21 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>144.9</v>
+        <v>130.9</v>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Heartleaf Pore Control Cleansing Oil</t>
+          <t>Invisible Glow Finish Sunstick</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" s="4" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="I22" s="4" t="n"/>
       <c r="J22" t="inlineStr">
@@ -1674,7 +1678,7 @@
       </c>
       <c r="K22" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/heartleaf-pore-control-cleansing-oil-200ml</t>
+          <t>https://anua.us/products/invisible-glow-finish-sunstick-1</t>
         </is>
       </c>
       <c r="L22" s="2">
@@ -1689,12 +1693,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MB003811</t>
+          <t>MB003872</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Heartleaf Pore Control Cleansing Oil: óleo de limpeza para os poros 200 ml</t>
+          <t>Mineral Weightless Finish Sunscreen: protetor solar mineral FPS 50 50 ml</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1703,21 +1707,21 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>159.9</v>
+        <v>130.9</v>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Heartleaf Pore Control Cleansing Oil</t>
+          <t>Mineral Weightless Finish Sunscreen</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" s="4" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="I23" s="4" t="n"/>
       <c r="J23" t="inlineStr">
@@ -1727,7 +1731,7 @@
       </c>
       <c r="K23" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/heartleaf-pore-control-cleansing-oil-200ml</t>
+          <t>https://anua.us/products/mineral-weightless-finish-sunscreen</t>
         </is>
       </c>
       <c r="L23" s="2">
@@ -1742,12 +1746,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>MB003871</t>
+          <t>MB003835</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Invisible Glow Finish Sunstick: protetor solar em bastão FPS 50 17,5 g</t>
+          <t>Niacinamide 5 TXA Brightening Pad: discos iluminadores (60 unidades)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1756,21 +1760,21 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>130.9</v>
+        <v>166.9</v>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Invisible Glow Finish Sunstick</t>
+          <t>Niacinamide 5 TXA Brightening Pad</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" s="4" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="I24" s="4" t="n"/>
       <c r="J24" t="inlineStr">
@@ -1780,7 +1784,7 @@
       </c>
       <c r="K24" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/invisible-glow-finish-sunstick-1</t>
+          <t>https://anua.us/products/niacinamide-5-txa-brightening-pad</t>
         </is>
       </c>
       <c r="L24" s="2">
@@ -1795,12 +1799,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MB003872</t>
+          <t>MB003859</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Mineral Weightless Finish Sunscreen: protetor solar mineral FPS 50 50 ml</t>
+          <t>PDRN 100 Hyaluronic Acid Booster Toner: tônico hidratante de PDRN 250 ml</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1809,21 +1813,21 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>130.9</v>
+        <v>152.9</v>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Mineral Weightless Finish Sunscreen</t>
+          <t>PDRN 100 Hyaluronic Acid Booster Toner</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" s="4" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="I25" s="4" t="n"/>
       <c r="J25" t="inlineStr">
@@ -1833,7 +1837,7 @@
       </c>
       <c r="K25" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/mineral-weightless-finish-sunscreen</t>
+          <t>https://anua.us/products/pdrn-100-hyaluronic-acid-booster-toner-1</t>
         </is>
       </c>
       <c r="L25" s="2">
@@ -1848,12 +1852,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>MB003814</t>
+          <t>MB003834</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Nano Retinol 0,3% + Niacin Renewing Serum: sérum de retinol e niacinamida 30 ml</t>
+          <t>PDRN 100 Hyaluronic Acid Glow Pad: discos hidratantes de PDRN (60 unidades)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1862,21 +1866,21 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>181.9</v>
+        <v>166.9</v>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Nano Retinol 0.3% + Niacin Renewing Serum</t>
+          <t>PDRN 100 Hyaluronic Acid Glow Pad</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" s="4" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I26" s="4" t="n"/>
       <c r="J26" t="inlineStr">
@@ -1886,7 +1890,7 @@
       </c>
       <c r="K26" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/nano-retinol-0-3-niacin-renewing-serum-1</t>
+          <t>https://anua.us/products/pdrn-100-hyaluronic-acid-glow-pad-1</t>
         </is>
       </c>
       <c r="L26" s="2">
@@ -1901,12 +1905,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>MB002695</t>
+          <t>MB003853</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Niacinamide 10 TXA 4 Serum: sérum para manchas e luminosidade 30 ml</t>
+          <t>PDRN Glow Boost Full Routine Set: rotina completa de PDRN em 7 produtos</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1915,23 +1919,25 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>174.9</v>
+        <v>1821.9</v>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Niacinamide 10 TXA 4 Serum for Brightening and Dark Spots</t>
+          <t>PDRN Glow Boost Full Routine Set</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="I27" s="4" t="n"/>
+        <v>220</v>
+      </c>
+      <c r="I27" s="4" t="n">
+        <v>333.8</v>
+      </c>
       <c r="J27" t="inlineStr">
         <is>
           <t>Sim</t>
@@ -1939,7 +1945,7 @@
       </c>
       <c r="K27" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/niacinamide-10-txa-4-serum-copy-1</t>
+          <t>https://anua.us/products/pdrn-glow-boost-full-routine-set</t>
         </is>
       </c>
       <c r="L27" s="2">
@@ -1954,12 +1960,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>MB003835</t>
+          <t>MB002681</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Niacinamide 5 TXA Brightening Pad: discos iluminadores (60 unidades)</t>
+          <t>PDRN Hyaluronic Acid 100 Moisturizing Cream: creme hidratante de PDRN 60 ml</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1968,21 +1974,21 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>166.9</v>
+        <v>225.9</v>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Niacinamide 5 TXA Brightening Pad</t>
+          <t>PDRN Hyaluronic Acid 100 Moisturizing Cream</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" s="4" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="I28" s="4" t="n"/>
       <c r="J28" t="inlineStr">
@@ -1992,7 +1998,7 @@
       </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/niacinamide-5-txa-brightening-pad</t>
+          <t>https://anua.us/products/pdrn-hyaluronic-acid-100-moisturizing-cream-1</t>
         </is>
       </c>
       <c r="L28" s="2">
@@ -2007,12 +2013,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>MB003848</t>
+          <t>MB003862</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Niacinamide TXA Brightening Booster Toner: tônico iluminador 250 ml</t>
+          <t>PDRN Hyaluronic Acid Moisturizing Cleansing Foam: espuma de limpeza hidratante 150 ml</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2021,21 +2027,21 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>152.9</v>
+        <v>108.9</v>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Niacinamide Tranexamic Acid Brightening Booster Toner</t>
+          <t>PDRN Hyaluronic Acid Moisturizing Cleansing Foam</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" s="4" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="I29" s="4" t="n"/>
       <c r="J29" t="inlineStr">
@@ -2045,7 +2051,7 @@
       </c>
       <c r="K29" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/niacinamide-tranexamic-acid-brightening-booster-toner-1</t>
+          <t>https://anua.us/products/pdrn-hyaluronic-acid-moisturizing-cleansing-foam</t>
         </is>
       </c>
       <c r="L29" s="2">
@@ -2060,12 +2066,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>MB003859</t>
+          <t>MB003861</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PDRN 100 Hyaluronic Acid Booster Toner: tônico hidratante de PDRN 250 ml</t>
+          <t>PDRN Lip Serum: sérum labial hidratante com PDRN 10 ml</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2074,21 +2080,21 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>152.9</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>PDRN 100 Hyaluronic Acid Booster Toner</t>
+          <t>PDRN Lip Serum</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" s="4" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="I30" s="4" t="n"/>
       <c r="J30" t="inlineStr">
@@ -2098,7 +2104,7 @@
       </c>
       <c r="K30" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/pdrn-100-hyaluronic-acid-booster-toner-1</t>
+          <t>https://anua.us/products/pdrn-lip-serum</t>
         </is>
       </c>
       <c r="L30" s="2">
@@ -2113,12 +2119,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>MB003834</t>
+          <t>MB002675</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PDRN 100 Hyaluronic Acid Glow Pad: discos hidratantes de PDRN (60 unidades)</t>
+          <t>PDRN Plump &amp; Dewy Glow Set: sérum em spray + creme com PDRN · Basic Set</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2127,21 +2133,25 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>166.9</v>
+        <v>663.9</v>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>PDRN 100 Hyaluronic Acid Glow Pad</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr"/>
+          <t>PDRN Plump &amp; Dewy Glow Set</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Basic Set</t>
+        </is>
+      </c>
       <c r="H31" s="4" t="n">
-        <v>23</v>
+        <v>91</v>
       </c>
       <c r="I31" s="4" t="n"/>
       <c r="J31" t="inlineStr">
@@ -2151,7 +2161,7 @@
       </c>
       <c r="K31" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/pdrn-100-hyaluronic-acid-glow-pad-1</t>
+          <t>https://anua.us/products/pdrn-all-day-dewy-glow-set?variant=51405018038550</t>
         </is>
       </c>
       <c r="L31" s="2">
@@ -2166,12 +2176,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>MB003876</t>
+          <t>MB002674</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>PDRN Collagen Glow Facial Serum Spray: bruma sérum com PDRN e colágeno 100 ml</t>
+          <t>PDRN Plump &amp; Dewy Glow Set: sérum em spray + creme com PDRN · Special Value Set</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2180,21 +2190,25 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>210.9</v>
+        <v>765.9</v>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>PDRN Collagen Glow Facial Serum Spray</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr"/>
+          <t>PDRN Plump &amp; Dewy Glow Set</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Basic Set</t>
+        </is>
+      </c>
       <c r="H32" s="4" t="n">
-        <v>29</v>
+        <v>91</v>
       </c>
       <c r="I32" s="4" t="n"/>
       <c r="J32" t="inlineStr">
@@ -2204,7 +2218,7 @@
       </c>
       <c r="K32" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/pdrn-100-hyaluronic-acid-hydrating-capsule-mist-100ml-1</t>
+          <t>https://anua.us/products/pdrn-all-day-dewy-glow-set?variant=51405018038550</t>
         </is>
       </c>
       <c r="L32" s="2">
@@ -2219,12 +2233,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>MB003853</t>
+          <t>MB003810</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PDRN Glow Boost Full Routine Set: rotina completa de PDRN em 7 produtos</t>
+          <t>Peach 70% Niacinamide Serum: sérum de pêssego e niacinamida 30 ml</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2233,25 +2247,23 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>1821.9</v>
+        <v>159.9</v>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>PDRN Glow Boost Full Routine Set</t>
+          <t>Peach 70% Niacinamide Serum</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" s="4" t="n">
-        <v>220</v>
-      </c>
-      <c r="I33" s="4" t="n">
-        <v>333.8</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="I33" s="4" t="n"/>
       <c r="J33" t="inlineStr">
         <is>
           <t>Sim</t>
@@ -2259,7 +2271,7 @@
       </c>
       <c r="K33" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/pdrn-glow-boost-full-routine-set</t>
+          <t>https://anua.us/products/peach-70-niacinamide-serum-copy</t>
         </is>
       </c>
       <c r="L33" s="2">
@@ -2274,12 +2286,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>MB002681</t>
+          <t>MB003846</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>PDRN Hyaluronic Acid 100 Moisturizing Cream: creme hidratante de PDRN 60 ml</t>
+          <t>Peach 77 Niacin Conditioning Milk: loção leitosa de pêssego 150 ml</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2288,21 +2300,21 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>225.9</v>
+        <v>181.9</v>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>PDRN Hyaluronic Acid 100 Moisturizing Cream</t>
+          <t>Peach 77 Niacin Conditioning Milk</t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" s="4" t="n">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="I34" s="4" t="n"/>
       <c r="J34" t="inlineStr">
@@ -2312,7 +2324,7 @@
       </c>
       <c r="K34" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/pdrn-hyaluronic-acid-100-moisturizing-cream-1</t>
+          <t>https://anua.us/products/peach-77-niacin-conditioning-milk</t>
         </is>
       </c>
       <c r="L34" s="2">
@@ -2327,12 +2339,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>MB003862</t>
+          <t>MB003824</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PDRN Hyaluronic Acid Moisturizing Cleansing Foam: espuma de limpeza hidratante 150 ml</t>
+          <t>Peach 77 Niacin Enriched Cream: creme de pêssego e niacinamida 50 ml</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2341,21 +2353,21 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>108.9</v>
+        <v>188.9</v>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>PDRN Hyaluronic Acid Moisturizing Cleansing Foam</t>
+          <t>Peach 77 Niacin Enriched Cream</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" s="4" t="n">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="I35" s="4" t="n"/>
       <c r="J35" t="inlineStr">
@@ -2365,7 +2377,7 @@
       </c>
       <c r="K35" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/pdrn-hyaluronic-acid-moisturizing-cleansing-foam</t>
+          <t>https://anua.us/products/peach-77-niacin-enriched-cream-1</t>
         </is>
       </c>
       <c r="L35" s="2">
@@ -2380,12 +2392,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>MB003861</t>
+          <t>MB003816</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>PDRN Lip Serum: sérum labial hidratante com PDRN 10 ml</t>
+          <t>Rice 70 Glow Milky Toner: tônico leitoso de arroz 250 ml</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2394,21 +2406,21 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>86.90000000000001</v>
+        <v>166.9</v>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>PDRN Lip Serum</t>
+          <t>Rice 70 Glow Milky Toner</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" s="4" t="n">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="I36" s="4" t="n"/>
       <c r="J36" t="inlineStr">
@@ -2418,7 +2430,7 @@
       </c>
       <c r="K36" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/pdrn-lip-serum</t>
+          <t>https://anua.us/products/rice-70-glow-milky-toner-copy</t>
         </is>
       </c>
       <c r="L36" s="2">
@@ -2433,12 +2445,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>MB002675</t>
+          <t>MB003831</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>PDRN Plump &amp; Dewy Glow Set: sérum em spray + creme com PDRN · Basic Set</t>
+          <t>Rice 70 Intensive Moisturizing Milk: loção hidratante de arroz 150 ml</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2447,25 +2459,21 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>663.9</v>
+        <v>144.9</v>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>PDRN Plump &amp; Dewy Glow Set</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>Basic Set</t>
-        </is>
-      </c>
+          <t>Rice 70 Intensive Moisturizing Milk</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
       <c r="H37" s="4" t="n">
-        <v>91</v>
+        <v>20</v>
       </c>
       <c r="I37" s="4" t="n"/>
       <c r="J37" t="inlineStr">
@@ -2475,7 +2483,7 @@
       </c>
       <c r="K37" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/pdrn-all-day-dewy-glow-set?variant=51405018038550</t>
+          <t>https://anua.us/products/rice-70-intensive-moisturizing-milk</t>
         </is>
       </c>
       <c r="L37" s="2">
@@ -2490,12 +2498,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>MB002674</t>
+          <t>MB003819</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>PDRN Plump &amp; Dewy Glow Set: sérum em spray + creme com PDRN · Special Value Set</t>
+          <t>Rice Ceramide 7 Hydrating Barrier Serum: sérum de arroz e ceramida 50 ml</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2504,25 +2512,21 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>765.9</v>
+        <v>166.9</v>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>PDRN Plump &amp; Dewy Glow Set</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>Basic Set</t>
-        </is>
-      </c>
+          <t>Rice Ceramide 7 Hydrating Barrier Serum</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
       <c r="H38" s="4" t="n">
-        <v>91</v>
+        <v>23</v>
       </c>
       <c r="I38" s="4" t="n"/>
       <c r="J38" t="inlineStr">
@@ -2532,7 +2536,7 @@
       </c>
       <c r="K38" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/pdrn-all-day-dewy-glow-set?variant=51405018038550</t>
+          <t>https://anua.us/products/rice-ceramide-7-hydrating-barrier-serum</t>
         </is>
       </c>
       <c r="L38" s="2">
@@ -2547,12 +2551,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>MB003810</t>
+          <t>MB003818</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Peach 70% Niacinamide Serum: sérum de pêssego e niacinamida 30 ml</t>
+          <t>Rice Enzyme Brightening Cleansing Powder: pó de limpeza enzimático de arroz 40 g</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2561,21 +2565,21 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>159.9</v>
+        <v>144.9</v>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Peach 70% Niacinamide Serum</t>
+          <t>Rice Enzyme Brightening Cleansing Powder</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" s="4" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I39" s="4" t="n"/>
       <c r="J39" t="inlineStr">
@@ -2585,7 +2589,7 @@
       </c>
       <c r="K39" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/peach-70-niacinamide-serum-copy</t>
+          <t>https://anua.us/products/rice-enzyme-brightening-cleansing-powder-1</t>
         </is>
       </c>
       <c r="L39" s="2">
@@ -2600,12 +2604,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>MB003846</t>
+          <t>MB003829</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Peach 77 Niacin Conditioning Milk: loção leitosa de pêssego 150 ml</t>
+          <t>Ultra-Thin Spot Cover Patch: adesivos invisíveis para espinhas (75 unidades)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2614,21 +2618,21 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>181.9</v>
+        <v>123.9</v>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Peach 77 Niacin Conditioning Milk</t>
+          <t>Ultra-Thin Spot Cover Patch</t>
         </is>
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" s="4" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="I40" s="4" t="n"/>
       <c r="J40" t="inlineStr">
@@ -2638,7 +2642,7 @@
       </c>
       <c r="K40" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/peach-77-niacin-conditioning-milk</t>
+          <t>https://anua.us/products/ultra-thin-spot-cover-patch</t>
         </is>
       </c>
       <c r="L40" s="2">
@@ -2653,12 +2657,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>MB003824</t>
+          <t>MB003864</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Peach 77 Niacin Enriched Cream: creme de pêssego e niacinamida 50 ml</t>
+          <t>Zero-cast Moisturizing Finish Sunscreen: protetor solar hidratante FPS 50 50 ml</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2667,21 +2671,21 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>188.9</v>
+        <v>131.9</v>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Peach 77 Niacin Enriched Cream</t>
+          <t>Zero-cast Moisturizing Finish Sunscreen</t>
         </is>
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" s="4" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="I41" s="4" t="n"/>
       <c r="J41" t="inlineStr">
@@ -2691,7 +2695,7 @@
       </c>
       <c r="K41" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/peach-77-niacin-enriched-cream-1</t>
+          <t>https://anua.us/products/zero-cast-moisturizing-finish-sunscreen</t>
         </is>
       </c>
       <c r="L41" s="2">
@@ -2706,39 +2710,37 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>MB003838</t>
+          <t>MB003808</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Peach Brightening Set: rotina iluminadora de pêssego e niacinamida em 4 passos</t>
+          <t>Heartleaf 77 Clear Pad</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>582.9</v>
+        <v>166.9</v>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Peach Brightening Set</t>
+          <t>Heartleaf 77 Clear Pad</t>
         </is>
       </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" s="4" t="n">
-        <v>80</v>
-      </c>
-      <c r="I42" s="4" t="n">
-        <v>85</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="I42" s="4" t="n"/>
       <c r="J42" t="inlineStr">
         <is>
           <t>Sim</t>
@@ -2746,7 +2748,7 @@
       </c>
       <c r="K42" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/peach-brightening-set</t>
+          <t>https://anua.us/products/heartleaf-77-toner-pad-160ml</t>
         </is>
       </c>
       <c r="L42" s="2">
@@ -2761,37 +2763,43 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>MB003816</t>
+          <t>MB003858</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Rice 70 Glow Milky Toner: tônico leitoso de arroz 250 ml</t>
+          <t>PDRN Collagen Wrinkle Smoothing Set</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>166.9</v>
+        <v>502.9</v>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Rice 70 Glow Milky Toner</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr"/>
+          <t>PDRN Collagen Wrinkle Smoothing Set</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Full Care Set</t>
+        </is>
+      </c>
       <c r="H43" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="I43" s="4" t="n"/>
+        <v>102</v>
+      </c>
+      <c r="I43" s="4" t="n">
+        <v>124</v>
+      </c>
       <c r="J43" t="inlineStr">
         <is>
           <t>Sim</t>
@@ -2799,7 +2807,7 @@
       </c>
       <c r="K43" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/rice-70-glow-milky-toner-copy</t>
+          <t>https://anua.us/products/pdrn-collagen-wrinkle-smoothing-intensive-set?variant=50904414585110</t>
         </is>
       </c>
       <c r="L43" s="2">
@@ -2814,35 +2822,35 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>MB003831</t>
+          <t>MB003854</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Rice 70 Intensive Moisturizing Milk: loção hidratante de arroz 150 ml</t>
+          <t>Revitalizing Eye Cream with 0.1% Retinol and Caffeine</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>144.9</v>
+        <v>166.9</v>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Rice 70 Intensive Moisturizing Milk</t>
+          <t>Retinol 0.1 Caffeine Revitalizing Eye Cream</t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" s="4" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="I44" s="4" t="n"/>
       <c r="J44" t="inlineStr">
@@ -2852,7 +2860,7 @@
       </c>
       <c r="K44" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/rice-70-intensive-moisturizing-milk</t>
+          <t>https://anua.us/products/retinol-0-1-caffeine-revitalizing-eye-cream</t>
         </is>
       </c>
       <c r="L44" s="2">
@@ -2867,35 +2875,35 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>MB003819</t>
+          <t>MB003865</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Rice Ceramide 7 Hydrating Barrier Serum: sérum de arroz e ceramida 50 ml</t>
+          <t>Soothing Moisturizer with Azelaic Acid and CICA</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>166.9</v>
+        <v>137.9</v>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Rice Ceramide 7 Hydrating Barrier Serum</t>
+          <t>Azelaic Acid CICA Skin Soothing Moisturizer</t>
         </is>
       </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" s="4" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I45" s="4" t="n"/>
       <c r="J45" t="inlineStr">
@@ -2905,7 +2913,7 @@
       </c>
       <c r="K45" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/rice-ceramide-7-hydrating-barrier-serum</t>
+          <t>https://anua.us/products/azelaic-acid-cica-skin-soothing-moisturizer</t>
         </is>
       </c>
       <c r="L45" s="2">
@@ -2920,35 +2928,35 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>MB003818</t>
+          <t>MB002726</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Rice Enzyme Brightening Cleansing Powder: pó de limpeza enzimático de arroz 40 g</t>
+          <t>Soothing Moisturizer with Azelaic Acid and CICA</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>144.9</v>
+        <v>137.9</v>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Provável — conferir</t>
+          <t>Certeiro</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Rice Enzyme Brightening Cleansing Powder</t>
+          <t>Azelaic Acid CICA Skin Soothing Moisturizer</t>
         </is>
       </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" s="4" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I46" s="4" t="n"/>
       <c r="J46" t="inlineStr">
@@ -2958,7 +2966,7 @@
       </c>
       <c r="K46" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/rice-enzyme-brightening-cleansing-powder-1</t>
+          <t>https://anua.us/products/azelaic-acid-cica-skin-soothing-moisturizer</t>
         </is>
       </c>
       <c r="L46" s="2">
@@ -2973,12 +2981,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>MB003856</t>
+          <t>MB003833</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Skin Recovery Duo: sérum de ácido azelaico 10% + creme de 3 ceramidas</t>
+          <t>Breakout Care Duo: sérum de ácido azelaico + creme localizado Heartleaf Centella</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2987,16 +2995,16 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>305.9</v>
-      </c>
-      <c r="E47" s="3" t="inlineStr">
+        <v>306.9</v>
+      </c>
+      <c r="E47" s="7" t="inlineStr">
         <is>
           <t>Provável — conferir</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Skin Recovery Duo</t>
+          <t>Breakout Care Duo</t>
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
@@ -3013,7 +3021,7 @@
       </c>
       <c r="K47" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/skin-recovery-duo</t>
+          <t>https://anua.us/products/intensive-spot-care-duo</t>
         </is>
       </c>
       <c r="L47" s="2">
@@ -3028,12 +3036,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>MB003829</t>
+          <t>MB003821</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Ultra-Thin Spot Cover Patch: adesivos invisíveis para espinhas (75 unidades)</t>
+          <t>Heartleaf Pore Cleansing Oil Mild: óleo de limpeza suave sem fragrância 200 ml</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -3042,21 +3050,21 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>123.9</v>
-      </c>
-      <c r="E48" s="3" t="inlineStr">
+        <v>144.9</v>
+      </c>
+      <c r="E48" s="7" t="inlineStr">
         <is>
           <t>Provável — conferir</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Ultra-Thin Spot Cover Patch</t>
+          <t>Heartleaf Pore Control Cleansing Oil</t>
         </is>
       </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" s="4" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="I48" s="4" t="n"/>
       <c r="J48" t="inlineStr">
@@ -3066,7 +3074,7 @@
       </c>
       <c r="K48" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/ultra-thin-spot-cover-patch</t>
+          <t>https://anua.us/products/heartleaf-pore-control-cleansing-oil-200ml</t>
         </is>
       </c>
       <c r="L48" s="2">
@@ -3081,12 +3089,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>MB003864</t>
+          <t>MB003814</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Zero-cast Moisturizing Finish Sunscreen: protetor solar hidratante FPS 50 50 ml</t>
+          <t>Nano Retinol 0,3% + Niacin Renewing Serum: sérum de retinol e niacinamida 30 ml</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -3095,21 +3103,21 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>131.9</v>
-      </c>
-      <c r="E49" s="3" t="inlineStr">
+        <v>181.9</v>
+      </c>
+      <c r="E49" s="7" t="inlineStr">
         <is>
           <t>Provável — conferir</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Zero-cast Moisturizing Finish Sunscreen</t>
+          <t>Nano Retinol 0.3% + Niacin Renewing Serum</t>
         </is>
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" s="4" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="I49" s="4" t="n"/>
       <c r="J49" t="inlineStr">
@@ -3119,7 +3127,7 @@
       </c>
       <c r="K49" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/zero-cast-moisturizing-finish-sunscreen</t>
+          <t>https://anua.us/products/nano-retinol-0-3-niacin-renewing-serum-1</t>
         </is>
       </c>
       <c r="L49" s="2">
@@ -3134,35 +3142,35 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>MB003808</t>
+          <t>MB002695</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Heartleaf 77 Clear Pad</t>
+          <t>Niacinamide 10 TXA 4 Serum: sérum para manchas e luminosidade 30 ml</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>166.9</v>
-      </c>
-      <c r="E50" s="3" t="inlineStr">
+        <v>174.9</v>
+      </c>
+      <c r="E50" s="7" t="inlineStr">
         <is>
           <t>Provável — conferir</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Heartleaf 77 Clear Pad</t>
+          <t>Niacinamide 10 TXA 4 Serum for Brightening and Dark Spots</t>
         </is>
       </c>
       <c r="G50" t="inlineStr"/>
       <c r="H50" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I50" s="4" t="n"/>
       <c r="J50" t="inlineStr">
@@ -3172,7 +3180,7 @@
       </c>
       <c r="K50" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/heartleaf-77-toner-pad-160ml</t>
+          <t>https://anua.us/products/niacinamide-10-txa-4-serum-copy-1</t>
         </is>
       </c>
       <c r="L50" s="2">
@@ -3187,35 +3195,35 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>MB003842</t>
+          <t>MB003848</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Hydrating Cleansing Foam with Hyaluronic Acid PDRN</t>
+          <t>Niacinamide TXA Brightening Booster Toner: tônico iluminador 250 ml</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>108.9</v>
-      </c>
-      <c r="E51" s="3" t="inlineStr">
+        <v>152.9</v>
+      </c>
+      <c r="E51" s="7" t="inlineStr">
         <is>
           <t>Provável — conferir</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>PDRN Hyaluronic Acid Moisturizing Cleansing Foam</t>
+          <t>Niacinamide Tranexamic Acid Brightening Booster Toner</t>
         </is>
       </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" s="4" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="I51" s="4" t="n"/>
       <c r="J51" t="inlineStr">
@@ -3225,7 +3233,7 @@
       </c>
       <c r="K51" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/pdrn-hyaluronic-acid-moisturizing-cleansing-foam</t>
+          <t>https://anua.us/products/niacinamide-tranexamic-acid-brightening-booster-toner-1</t>
         </is>
       </c>
       <c r="L51" s="2">
@@ -3240,35 +3248,35 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>MB003875</t>
+          <t>MB003876</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Mini Spray Sérum Facial PDRN Colágeno Glow</t>
+          <t>PDRN Collagen Glow Facial Serum Spray: bruma sérum com PDRN e colágeno 100 ml</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>144.9</v>
-      </c>
-      <c r="E52" s="3" t="inlineStr">
+        <v>210.9</v>
+      </c>
+      <c r="E52" s="7" t="inlineStr">
         <is>
           <t>Provável — conferir</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>PDRN Collagen Glow Facial Serum Spray Mini</t>
+          <t>PDRN Collagen Glow Facial Serum Spray</t>
         </is>
       </c>
       <c r="G52" t="inlineStr"/>
       <c r="H52" s="4" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="I52" s="4" t="n"/>
       <c r="J52" t="inlineStr">
@@ -3278,7 +3286,7 @@
       </c>
       <c r="K52" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/pdrn-collagen-glow-facial-serum-spray-mini</t>
+          <t>https://anua.us/products/pdrn-100-hyaluronic-acid-hydrating-capsule-mist-100ml-1</t>
         </is>
       </c>
       <c r="L52" s="2">
@@ -3293,42 +3301,38 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>MB003858</t>
+          <t>MB003838</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>PDRN Collagen Wrinkle Smoothing Set</t>
+          <t>Peach Brightening Set: rotina iluminadora de pêssego e niacinamida em 4 passos</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>502.9</v>
-      </c>
-      <c r="E53" s="3" t="inlineStr">
+        <v>582.9</v>
+      </c>
+      <c r="E53" s="7" t="inlineStr">
         <is>
           <t>Provável — conferir</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>PDRN Collagen Wrinkle Smoothing Set</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>Full Care Set</t>
-        </is>
-      </c>
+          <t>Peach Brightening Set</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr"/>
       <c r="H53" s="4" t="n">
-        <v>102</v>
+        <v>80</v>
       </c>
       <c r="I53" s="4" t="n">
-        <v>124</v>
+        <v>85</v>
       </c>
       <c r="J53" t="inlineStr">
         <is>
@@ -3337,7 +3341,7 @@
       </c>
       <c r="K53" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/pdrn-collagen-wrinkle-smoothing-intensive-set?variant=50904414585110</t>
+          <t>https://anua.us/products/peach-brightening-set</t>
         </is>
       </c>
       <c r="L53" s="2">
@@ -3352,38 +3356,38 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>MB003868</t>
+          <t>MB003856</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>PDRN Glow Boost: Kit Completo de Rotina</t>
+          <t>Skin Recovery Duo: sérum de ácido azelaico 10% + creme de 3 ceramidas</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>1821.9</v>
-      </c>
-      <c r="E54" s="3" t="inlineStr">
+        <v>305.9</v>
+      </c>
+      <c r="E54" s="7" t="inlineStr">
         <is>
           <t>Provável — conferir</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>PDRN Glow Boost Full Routine Set</t>
+          <t>Skin Recovery Duo</t>
         </is>
       </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" s="4" t="n">
-        <v>220</v>
+        <v>42</v>
       </c>
       <c r="I54" s="4" t="n">
-        <v>333.8</v>
+        <v>50</v>
       </c>
       <c r="J54" t="inlineStr">
         <is>
@@ -3392,7 +3396,7 @@
       </c>
       <c r="K54" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/pdrn-glow-boost-full-routine-set</t>
+          <t>https://anua.us/products/skin-recovery-duo</t>
         </is>
       </c>
       <c r="L54" s="2">
@@ -3407,12 +3411,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>MB003854</t>
+          <t>MB003842</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Revitalizing Eye Cream with 0.1% Retinol and Caffeine</t>
+          <t>Hydrating Cleansing Foam with Hyaluronic Acid PDRN</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -3421,21 +3425,21 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>166.9</v>
-      </c>
-      <c r="E55" s="3" t="inlineStr">
+        <v>108.9</v>
+      </c>
+      <c r="E55" s="7" t="inlineStr">
         <is>
           <t>Provável — conferir</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Retinol 0.1 Caffeine Revitalizing Eye Cream</t>
+          <t>PDRN Hyaluronic Acid Moisturizing Cleansing Foam</t>
         </is>
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" s="4" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="I55" s="4" t="n"/>
       <c r="J55" t="inlineStr">
@@ -3445,7 +3449,7 @@
       </c>
       <c r="K55" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/retinol-0-1-caffeine-revitalizing-eye-cream</t>
+          <t>https://anua.us/products/pdrn-hyaluronic-acid-moisturizing-cleansing-foam</t>
         </is>
       </c>
       <c r="L55" s="2">
@@ -3460,12 +3464,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>MB003865</t>
+          <t>MB003875</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Soothing Moisturizer with Azelaic Acid and CICA</t>
+          <t>Mini Spray Sérum Facial PDRN Colágeno Glow</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -3474,21 +3478,21 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>137.9</v>
-      </c>
-      <c r="E56" s="3" t="inlineStr">
+        <v>144.9</v>
+      </c>
+      <c r="E56" s="7" t="inlineStr">
         <is>
           <t>Provável — conferir</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Azelaic Acid CICA Skin Soothing Moisturizer</t>
+          <t>PDRN Collagen Glow Facial Serum Spray Mini</t>
         </is>
       </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I56" s="4" t="n"/>
       <c r="J56" t="inlineStr">
@@ -3498,7 +3502,7 @@
       </c>
       <c r="K56" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/azelaic-acid-cica-skin-soothing-moisturizer</t>
+          <t>https://anua.us/products/pdrn-collagen-glow-facial-serum-spray-mini</t>
         </is>
       </c>
       <c r="L56" s="2">
@@ -3513,12 +3517,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>MB002726</t>
+          <t>MB003868</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Soothing Moisturizer with Azelaic Acid and CICA</t>
+          <t>PDRN Glow Boost: Kit Completo de Rotina</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -3527,23 +3531,25 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>137.9</v>
-      </c>
-      <c r="E57" s="3" t="inlineStr">
+        <v>1821.9</v>
+      </c>
+      <c r="E57" s="7" t="inlineStr">
         <is>
           <t>Provável — conferir</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Azelaic Acid CICA Skin Soothing Moisturizer</t>
+          <t>PDRN Glow Boost Full Routine Set</t>
         </is>
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="I57" s="4" t="n"/>
+        <v>220</v>
+      </c>
+      <c r="I57" s="4" t="n">
+        <v>333.8</v>
+      </c>
       <c r="J57" t="inlineStr">
         <is>
           <t>Sim</t>
@@ -3551,7 +3557,7 @@
       </c>
       <c r="K57" s="5" t="inlineStr">
         <is>
-          <t>https://anua.us/products/azelaic-acid-cica-skin-soothing-moisturizer</t>
+          <t>https://anua.us/products/pdrn-glow-boost-full-routine-set</t>
         </is>
       </c>
       <c r="L57" s="2">
@@ -3582,7 +3588,7 @@
       <c r="D58" s="2" t="n">
         <v>152.9</v>
       </c>
-      <c r="E58" s="7" t="inlineStr">
+      <c r="E58" s="8" t="inlineStr">
         <is>
           <t>Conferir (tamanho/kit diferente)</t>
         </is>
@@ -3635,7 +3641,7 @@
       <c r="D59" s="2" t="n">
         <v>144.9</v>
       </c>
-      <c r="E59" s="7" t="inlineStr">
+      <c r="E59" s="8" t="inlineStr">
         <is>
           <t>Conferir (tamanho/kit diferente)</t>
         </is>
@@ -3688,7 +3694,7 @@
       <c r="D60" s="2" t="n">
         <v>144.9</v>
       </c>
-      <c r="E60" s="7" t="inlineStr">
+      <c r="E60" s="8" t="inlineStr">
         <is>
           <t>Conferir (tamanho/kit diferente)</t>
         </is>
@@ -3741,7 +3747,7 @@
       <c r="D61" s="2" t="n">
         <v>159.9</v>
       </c>
-      <c r="E61" s="7" t="inlineStr">
+      <c r="E61" s="8" t="inlineStr">
         <is>
           <t>Conferir (tamanho/kit diferente)</t>
         </is>
@@ -3794,7 +3800,7 @@
       <c r="D62" s="2" t="n">
         <v>159.9</v>
       </c>
-      <c r="E62" s="7" t="inlineStr">
+      <c r="E62" s="8" t="inlineStr">
         <is>
           <t>Conferir (tamanho/kit diferente)</t>
         </is>
@@ -3847,7 +3853,7 @@
       <c r="D63" s="2" t="n">
         <v>152.9</v>
       </c>
-      <c r="E63" s="7" t="inlineStr">
+      <c r="E63" s="8" t="inlineStr">
         <is>
           <t>Conferir (tamanho/kit diferente)</t>
         </is>
@@ -3900,7 +3906,7 @@
       <c r="D64" s="2" t="n">
         <v>437.9</v>
       </c>
-      <c r="E64" s="7" t="inlineStr">
+      <c r="E64" s="8" t="inlineStr">
         <is>
           <t>Conferir (tamanho/kit diferente)</t>
         </is>
@@ -3953,7 +3959,7 @@
       <c r="D65" s="2" t="n">
         <v>844.9</v>
       </c>
-      <c r="E65" s="7" t="inlineStr">
+      <c r="E65" s="8" t="inlineStr">
         <is>
           <t>Fraco — conferir</t>
         </is>
@@ -4008,7 +4014,7 @@
       <c r="D66" s="2" t="n">
         <v>159.9</v>
       </c>
-      <c r="E66" s="7" t="inlineStr">
+      <c r="E66" s="8" t="inlineStr">
         <is>
           <t>Fraco — conferir</t>
         </is>
@@ -4061,7 +4067,7 @@
       <c r="D67" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="E67" s="7" t="inlineStr">
+      <c r="E67" s="8" t="inlineStr">
         <is>
           <t>Fraco — conferir</t>
         </is>
@@ -4116,7 +4122,7 @@
       <c r="D68" s="2" t="n">
         <v>152.9</v>
       </c>
-      <c r="E68" s="7" t="inlineStr">
+      <c r="E68" s="8" t="inlineStr">
         <is>
           <t>Fraco — conferir</t>
         </is>
@@ -8737,7 +8743,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Site oficial: https://anua.us · loja "Anua US" · moeda USD · lido em 30/10/2026 06:02 UTC</t>
+          <t>Site oficial: https://anua.us · loja "Anua US" · moeda USD · lido em 30/10/2026 06:03 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>